<commit_message>
feat: support international product pricing
</commit_message>
<xml_diff>
--- a/public/templates/street-culture-product-import.xlsx
+++ b/public/templates/street-culture-product-import.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRODUCTS" sheetId="1" r:id="R68b7ec54783349f9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VARIANTS" sheetId="2" r:id="Rb94d21819c934a20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MEDIA" sheetId="3" r:id="R27f60eae117642b8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCTIONS" sheetId="4" r:id="R5e52d1945f4b4dea"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REFERENCE VALUES" sheetId="5" r:id="R0965fa62dd234066"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRODUCTS" sheetId="1" r:id="R5080bdf697484912"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VARIANTS" sheetId="2" r:id="R03eff53b82d743d3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MEDIA" sheetId="3" r:id="R19cbf145e9884fd0"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCTIONS" sheetId="4" r:id="Rd9a3dbf9060d49b3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REFERENCE VALUES" sheetId="5" r:id="R69146d8685e042bf"/>
   </sheets>
 </workbook>
 </file>
@@ -512,7 +512,7 @@
         <v>Required variant fields</v>
       </c>
       <c r="B5" t="str">
-        <v>product_reference, size, size_system, quantity = 1; one variant row per size.</v>
+        <v>Required: product_reference, size, size_system, quantity = 1, and active = TRUE. Optional price_override uses the same currency as the matching PRODUCTS row.</v>
       </c>
     </row>
     <row r="6">
@@ -520,7 +520,7 @@
         <v>Currency</v>
       </c>
       <c r="B6" t="str">
-        <v>Use MZN for store-owned inventory. Checkout through M-Pesa charges MZN.</v>
+        <v>Use MZN, USD, EUR, ZAR, or GBP. Foreign prices are converted to MZN during preview using one recorded daily rate. Review the MZN amount before confirming; M-Pesa charges MZN.</v>
       </c>
     </row>
     <row r="7">

</xml_diff>